<commit_message>
Update models to clarify Google One bulk pricing and adopt illustrative unit economics phrasing
</commit_message>
<xml_diff>
--- a/Altura_Detailed_Convergence_Feasibility_Model.xlsx
+++ b/Altura_Detailed_Convergence_Feasibility_Model.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Financial &amp; Strategic Justification</t>
+          <t>Illustrative Modeling &amp; Strategic Justification</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Financial Feasibility: Churn-Driven LTV Multipliers &amp; High-Return Cohort Economics</t>
+          <t>Illustrative Financial Feasibility (Based on industry benchmarks and internal modeling assumptions)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
@@ -977,6 +977,7 @@
  - Outbound MNP CAC: ₹1,530/customer (₹500 switcher rebate, labor, runner delivery, tech commission, local marketing).
 2. Detailed Operating &amp; Return Economics:
  - Recurring monthly Opex: ₹535/mo per user (bandwidth, content licensing, cellular tower pool, Google bulk royalty, cloud storage, bank administration).
+ - Google One (200GB): Modeled as an assumed volume-negotiated enterprise licensing rate (wholesale bulk transfer pricing rather than retail).
  - Payback Period: The initial ₹6,330 hardware Capex + switcher CAC is fully recovered in 8.6 Months (inclusive of 3-mos promo ₹999/mo).
  - Weighted EBITDA Margin: 27.5% on standard ₹1,499/mo plan (yielding ₹914/mo EBITDA profit).
  - Churn Arbitrage LTV: Reducing churn from 22.0% (standalone) to 5.0% (triple-play) extends lifetime to 20 years, yielding ₹97,511 Net EBITDA LTV (4.82x multiplier) and 33.4x ROI.</t>
@@ -1005,18 +1006,18 @@
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="66" customWidth="1" min="5" max="5"/>
+    <col width="117" customWidth="1" min="5" max="5"/>
     <col width="77" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ALTURA HOUSEHOLD CONVERGENCE COMPREHENSIVE COST CATALOG</t>
+          <t>ILLUSTRATIVE UNIT ECONOMICS &amp; MODELING ASSUMPTIONS</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. ONE-TIME CAPITAL &amp; DEVELOPMENT COSTS (CAPEX)</t>
+          <t>1. ONE-TIME CAPITAL &amp; DEVELOPMENT COSTS (CAPEX - ASSUMED)</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1198,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2. ONE-TIME CUSTOMER ACQUISITION COSTS (CAC)</t>
+          <t>2. ONE-TIME CUSTOMER ACQUISITION COSTS (CAC - ASSUMED)</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1423,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>3. MONTHLY RECURRING OPERATIONAL COSTS (OPEX)</t>
+          <t>3. MONTHLY RECURRING OPERATIONAL COSTS (OPEX - ASSUMED)</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1570,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Wholesale bulk storage royalty fee paid directly to Google</t>
+          <t>Assumed volume-negotiated enterprise licensing cost (Airtel offers 100GB/6-mos; Altura negotiates 200GB wholesale)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Format Excel models to use only professional Airtel Red and bold white highlights
</commit_message>
<xml_diff>
--- a/Altura_Detailed_Convergence_Feasibility_Model.xlsx
+++ b/Altura_Detailed_Convergence_Feasibility_Model.xlsx
@@ -64,7 +64,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -75,30 +75,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00ED1D24"/>
         <bgColor rgb="00ED1D24"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ECFDF5"/>
-        <bgColor rgb="00ECFDF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0F7FA"/>
-        <bgColor rgb="00E0F7FA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -136,23 +112,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -161,84 +134,50 @@
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,21 +616,21 @@
       <c r="B5" s="5" t="n">
         <v>4800</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>4800</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="5" t="n">
         <v>3300</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="5" t="n">
         <v>3300</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Amortized asset base</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>ONT Router (₹1,500) + TV Box (₹1,800) + Camera (₹1,500); Segment B/C reuse existing router ONT</t>
         </is>
@@ -706,21 +645,21 @@
       <c r="B6" s="5" t="n">
         <v>1530</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="5" t="n">
         <v>1130</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>CAC cost savings</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Outbound requires ads, runner, tech commission &amp; ₹500 rebate; Segment B requires mobile MNP port-in</t>
         </is>
@@ -732,28 +671,28 @@
           <t>Total Upfront Investment per Subscriber</t>
         </is>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="8">
         <f>B5+B6</f>
         <v/>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="8">
         <f>C5+C6</f>
         <v/>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="8">
         <f>D5+D6</f>
         <v/>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="8">
         <f>E5+E6</f>
         <v/>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Initial layout per HH</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Combined CapEx + CAC absorbed by Altura to remove subscriber migration friction</t>
         </is>
@@ -768,21 +707,21 @@
       <c r="B8" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Waived for existing mobile</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>One-time contract buyout rebate credited on first bill; ₹0 for existing Altura mobile accounts</t>
         </is>
@@ -797,21 +736,21 @@
       <c r="B9" s="5" t="n">
         <v>949</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="5" t="n">
         <v>949</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="5" t="n">
         <v>949</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="5" t="n">
         <v>949</v>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>1.00x Promo ARPU</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>₹999 promotional price minus ₹50 Autopay discount (waived entry barrier)</t>
         </is>
@@ -826,21 +765,21 @@
       <c r="B10" s="5" t="n">
         <v>1449</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="5" t="n">
         <v>1449</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="5" t="n">
         <v>1449</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="5" t="n">
         <v>1449</v>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>1.12x ARPU increase</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>₹1,499 standard Family Secure price minus ₹50 Autopay discount</t>
         </is>
@@ -852,24 +791,24 @@
           <t>Weighted Recurring Monthly Opex</t>
         </is>
       </c>
-      <c r="B11" s="11" t="n">
+      <c r="B11" s="9" t="n">
         <v>535</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="9" t="n">
         <v>535</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="9" t="n">
         <v>535</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="9" t="n">
         <v>535</v>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Highly scalable network</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Includes bandwidth backhaul, postpaid pool, Google One, AWS camera cloud, bank, &amp; loyalty program</t>
         </is>
@@ -881,24 +820,24 @@
           <t>Monthly EBITDA Margin (Standard Period)</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="10" t="n">
         <v>0.6308</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="10" t="n">
         <v>0.6308</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="10" t="n">
         <v>0.6308</v>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="10" t="n">
         <v>0.6308</v>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>63.1% EBITDA Margin</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>High operating margin once initial customer-end hardware is capitalized and amortized</t>
         </is>
@@ -910,24 +849,24 @@
           <t>Average Customer Relationship (Years)</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>4.44x Churn Arbitrage</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Bundle reduces annual churn from 22.0% (standalone) to 5.0% (triple-play)</t>
         </is>
@@ -939,24 +878,24 @@
           <t>Payback Break-Even Period (Months)</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="12" t="n">
         <v>8.57</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="12" t="n">
         <v>7.33</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="12" t="n">
         <v>6.49</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="12" t="n">
         <v>5.69</v>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Saves up to 3.0 months</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Time to recover initial hardware subsidy + CAC outlay; existing base conversions pay back significantly faster</t>
         </is>
@@ -968,24 +907,24 @@
           <t>Net EBITDA Lifetime Value (LTV)</t>
         </is>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="8" t="n">
         <v>97511</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="8" t="n">
         <v>98411</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="8" t="n">
         <v>98411</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="8" t="n">
         <v>98411</v>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>4.82x EBITDA Multiplier</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Consolidated household LTV net of CAC vs. stand-alone mobile/broadband LTV (₹20,226)</t>
         </is>
@@ -997,24 +936,24 @@
           <t>Ecosystem Return on Investment (ROI)</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="13" t="n">
         <v>15.4</v>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="13" t="n">
         <v>18.9</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="13" t="n">
         <v>22.2</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="13" t="n">
         <v>26.6</v>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Up to 26.6x Lifetime return</t>
         </is>
       </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>EBITDA Lifetime contribution divided by total initial Capex + CAC outlay</t>
         </is>
@@ -1047,51 +986,51 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Slide 2: Solution Engine</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Inbound-First Base Conversion Strategy</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>Saves up to ₹2,630 in upfront router and SIM marketing CAC by targeting existing high-trust customers first.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>Slide 3: Financial Feasibility</t>
-        </is>
-      </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Slide 3: Feasibility</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Segment C Payback = 5.7 Months (ROI = 26.6x)</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>Consolidating existing double-play subscribers only requires a ₹3.7k TV/Camera outlay, returning ₹98k in lifetime EBITDA.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Slide 3: Financial Feasibility</t>
-        </is>
-      </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>Slide 3: Feasibility</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Average Base Payback = 6.5 Months</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Waiving upfront hardware and charging ₹999 promo price is highly feasible, recovering investments 2.1 months faster than outbound poaching.</t>
         </is>
@@ -1156,22 +1095,22 @@
       </c>
     </row>
     <row r="4" ht="200" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Slide 2: Solution</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Altura Home: The Strategy in Action (Organic Base Conversion + Outbound Poaching)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Leveraging organic single-play and double-play subscriber bases as the primary high-retention launch pad, while positioning outbound competitor poaching as a secondary future lever.</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. Focus on Converting Our Own Base First:
  - Inbound Cross-Selling: Target existing Mobile postpaid-only, Broadband-only, and standalone Double-Play customers to upgrade them to Family Secure.
@@ -1181,33 +1120,33 @@
  - Build-Your-Own-Bundle Customizer: Interactive calculator showing real-time monthly billing savings and Thanks Coins to dismantle Utility-Arbitrage Bias.
  - AirBot AI digital concierge to simplify profile matching and eliminate onboarding friction.
 3. Outbound Competitor Poaching (Secondary Future Lever):
- - Doorstep MNP in 15 Minutes: Eqquiping in-home installation technicians with mobile activation apps to execute MNP port-ins.
+ - Doorstep MNP in 15 Minutes: Equipping field service technicians (lowest CAC of ₹150 and lowest decay rate of 12%) with MNP activation apps to execute MNP port-ins.
  - Switcher's Contract Rebate: One-time ₹500 cashback credit to offset switcher penalty fees.</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Targeting our own base first eliminates the largest Capex and marketing CAC costs, securing maximum value before expanding outbound.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="200" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Slide 3: Feasibility</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Illustrative Financial Feasibility (Based on industry benchmarks and internal modeling assumptions)</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Amortizing upfront development, hardware subsidy, and switcher rebates through high-retention monthly recurring EBITDA margins.</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. Existing Base Conversion Economics (Highest Return Loop):
  - Segment A (Mobile-Only Base): Initial outlay ₹5,200 (Router/TV Box/Camera/Labor/Upsell) -&gt; Payback = 7.3 Months (ROI = 18.9x).
@@ -1220,9 +1159,9 @@
  - Churn Arbitrage LTV: Consolidating services reduces annual churn from 22.0% (standalone) to 5.0% (bundled), extending relationship lifetime from 4.5 to 20 years, yielding ₹98,411 Lifetime EBITDA contribution.</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>waiving hardware and contract buyout costs is highly feasible, returning the initial layouts in 5.7 to 7.3 months for our own base.</t>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>waiving upfront hardware and contract buyout costs is highly feasible, returning the initial layouts in 5.7 to 7.3 months for our own base.</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1238,7 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Website &amp; AI Portal Development</t>
         </is>
@@ -1313,19 +1252,19 @@
       <c r="D5" s="5" t="n">
         <v>2000000</v>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Amortized over first 1,000 cohort (₹2,000/HH)</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>Design, customizer custom frontend, AirBot AI NLP training, APIs</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Dual-Band ONT Wi-Fi Router</t>
         </is>
@@ -1339,19 +1278,19 @@
       <c r="D6" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Amortized over customer contract lifetime</t>
         </is>
       </c>
-      <c r="F6" s="21" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>Waived to eliminate migration barrier; high-speed home connectivity anchor</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Altura Xstream 4K Smart Android Box</t>
         </is>
@@ -1365,19 +1304,19 @@
       <c r="D7" s="5" t="n">
         <v>1800</v>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Amortized over customer contract lifetime</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>Waived; hybrid satellite/OTT television anchor to stop DTH revenue drop</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Altura Xsafe AI Smart Security Camera</t>
         </is>
@@ -1391,41 +1330,41 @@
       <c r="D8" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Amortized over customer contract lifetime</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>Waived; smart home security camera enlisting cell-failover backup tech</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Total Capex per Subscriber</t>
         </is>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="16">
         <f>SUM(B6:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="16">
         <f>SUM(C6:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="24">
+      <c r="D9" s="16">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="23" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>Hardware Subsidy</t>
         </is>
       </c>
-      <c r="F9" s="23" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Total Capex absorbed per Household</t>
         </is>
@@ -1472,7 +1411,7 @@
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Technician Labor Cost</t>
         </is>
@@ -1486,19 +1425,19 @@
       <c r="D13" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>In-Home Service Engineers</t>
         </is>
       </c>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="F13" s="14" t="inlineStr">
         <is>
           <t>Cost of initial physical visit and hardware deployment</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Physical SIM Card &amp; Security Chip</t>
         </is>
@@ -1512,19 +1451,19 @@
       <c r="D14" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Outbound Delivery</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>Provisioning costs for 2 family postpaid SIM cards</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>MNP Switcher Cashback (Rebate)</t>
         </is>
@@ -1538,19 +1477,19 @@
       <c r="D15" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Outbound MNP</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="14" t="inlineStr">
         <is>
           <t>Buyout penalty fee rebate given to Jio/Vi switcher on first bill</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Doorstep MNP Delivery Runner</t>
         </is>
@@ -1564,19 +1503,19 @@
       <c r="D16" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>Outbound Delivery</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Runner cost for doorstep delivery and SIM activation in 15 mins</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Technician MNP Porting Commission</t>
         </is>
@@ -1590,19 +1529,19 @@
       <c r="D17" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>In-Home Service Engineers</t>
         </is>
       </c>
-      <c r="F17" s="21" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Engineers get bonus incentive to check competitor SIMs and execute porting</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Blended Marketing/Advertising Spend</t>
         </is>
@@ -1616,41 +1555,41 @@
       <c r="D18" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>Digital Portal / OOH</t>
         </is>
       </c>
-      <c r="F18" s="21" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Pincode-targeted search ads, billboards, and performance marketing</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Total CAC per Subscriber</t>
         </is>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="16">
         <f>SUM(B13:B18)</f>
         <v/>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="16">
         <f>SUM(C13:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="24">
+      <c r="D19" s="16">
         <f>B19-C19</f>
         <v/>
       </c>
-      <c r="E19" s="23" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Ecosystem Outbound CAC</t>
         </is>
       </c>
-      <c r="F19" s="23" t="inlineStr">
+      <c r="F19" s="15" t="inlineStr">
         <is>
           <t>Total acquisition CAC outlay per customer</t>
         </is>
@@ -1697,7 +1636,7 @@
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Broadband Backhaul Bandwidth</t>
         </is>
@@ -1705,29 +1644,29 @@
       <c r="B23" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>Fiber Broadband</t>
         </is>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D23" s="14" t="inlineStr">
         <is>
           <t>Broadband (32% EBITDA)</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="14" t="inlineStr">
         <is>
           <t>Incremental bandwidth cost of laying and servicing fiber lines</t>
         </is>
       </c>
-      <c r="F23" s="21" t="inlineStr">
+      <c r="F23" s="14" t="inlineStr">
         <is>
           <t>Home fiber link connection backhaul and hardware maintenance</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Cellular Network Data Pool (2 SIMs)</t>
         </is>
@@ -1735,29 +1674,29 @@
       <c r="B24" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>Postpaid Mobile</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>Mobility (28% EBITDA)</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Core cellular tower maintenance and pool data routing</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>Postpaid cell pool, priority network routing slot</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>DTH Carriage &amp; Content Licensing</t>
         </is>
@@ -1765,29 +1704,29 @@
       <c r="B25" s="5" t="n">
         <v>120</v>
       </c>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Xstream Play TV</t>
         </is>
       </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>DTH / TV (12% EBITDA)</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Content carriage licensing fee paid to broadcasters/OTT players</t>
         </is>
       </c>
-      <c r="F25" s="21" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>4K TV feed, basic channels, carriage, and OTT app licenses</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Google One Bulk License Royalty</t>
         </is>
@@ -1795,29 +1734,29 @@
       <c r="B26" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>Google One (200GB)</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>N/A (Net 15% Margin)</t>
         </is>
       </c>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>Assumed volume-negotiated enterprise licensing cost (Airtel offers 100GB/6-mos; Altura negotiates 200GB wholesale)</t>
         </is>
       </c>
-      <c r="F26" s="21" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>200GB cloud storage space, family backup cloud access</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="21" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Xsafe Camera Cloud Storage Hosting</t>
         </is>
@@ -1825,29 +1764,29 @@
       <c r="B27" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="C27" s="21" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>Xsafe Smart Camera</t>
         </is>
       </c>
-      <c r="D27" s="21" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Surveillance (35% EBITDA)</t>
         </is>
       </c>
-      <c r="E27" s="21" t="inlineStr">
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>AWS/Azure cloud hosting cost per camera cloud recording feed</t>
         </is>
       </c>
-      <c r="F27" s="21" t="inlineStr">
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>7-day recording loop storage space and humanoid alert notification</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Payments Bank Administration Fee</t>
         </is>
@@ -1855,29 +1794,29 @@
       <c r="B28" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C28" s="21" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>Payments Bank</t>
         </is>
       </c>
-      <c r="D28" s="21" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Banking (50% EBITDA)</t>
         </is>
       </c>
-      <c r="E28" s="21" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Transaction clearing, database administration, and KYC cost</t>
         </is>
       </c>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>7% interest rate margin management, Safe Pay anti-fraud engine</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="21" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Thanks Coins Loyalty Redemption</t>
         </is>
@@ -1885,53 +1824,53 @@
       <c r="B29" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>Ecosystem Reward</t>
         </is>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>Ecosystem Loyalty</t>
         </is>
       </c>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="E29" s="14" t="inlineStr">
         <is>
           <t>Margin cost of coin redemptions at retail partner merchants</t>
         </is>
       </c>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Loyalty coins program, incentivizing Autopay and monthly renewals</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="25" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>Total Recurring Monthly Opex</t>
         </is>
       </c>
-      <c r="B30" s="26">
+      <c r="B30" s="16">
         <f>SUM(B23:B29)</f>
         <v/>
       </c>
-      <c r="C30" s="25" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Combined Services</t>
         </is>
       </c>
-      <c r="D30" s="25" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>Weighted Segments</t>
         </is>
       </c>
-      <c r="E30" s="25" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>EBITDA Profit Factor</t>
         </is>
       </c>
-      <c r="F30" s="25" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>Altura's total monthly operational cost per user</t>
         </is>
@@ -2022,45 +1961,45 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Month 0 (Upfront)</t>
         </is>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="18" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="19">
         <f>-B5*'Dashboard &amp; Summary'!C7</f>
         <v/>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="18" t="n">
         <v>1000</v>
       </c>
-      <c r="E5" s="29">
+      <c r="E5" s="19">
         <f>-D5*'Dashboard &amp; Summary'!D7</f>
         <v/>
       </c>
-      <c r="F5" s="28" t="n">
+      <c r="F5" s="18" t="n">
         <v>1000</v>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="19">
         <f>-F5*'Dashboard &amp; Summary'!E7</f>
         <v/>
       </c>
-      <c r="H5" s="30" t="inlineStr">
+      <c r="H5" s="20" t="inlineStr">
         <is>
           <t>Hardware subsidies + Digital Upsell labor</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="18">
         <f>B5*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2068,7 +2007,7 @@
         <f>C5+(B6*414)</f>
         <v/>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="18">
         <f>D5*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2076,7 +2015,7 @@
         <f>E5+(D6*414)</f>
         <v/>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="18">
         <f>F5*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2084,19 +2023,19 @@
         <f>G5+(F6*414)</f>
         <v/>
       </c>
-      <c r="H6" s="33" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹949 Net)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="B7" s="32">
+      <c r="B7" s="18">
         <f>B6*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2104,7 +2043,7 @@
         <f>C6+(B7*414)</f>
         <v/>
       </c>
-      <c r="D7" s="32">
+      <c r="D7" s="18">
         <f>D6*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2112,7 +2051,7 @@
         <f>E6+(D7*414)</f>
         <v/>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="18">
         <f>F6*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2120,19 +2059,19 @@
         <f>G6+(F7*414)</f>
         <v/>
       </c>
-      <c r="H7" s="33" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹949 Net)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="B8" s="32">
+      <c r="B8" s="18">
         <f>B7*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2140,7 +2079,7 @@
         <f>C7+(B8*414)</f>
         <v/>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="18">
         <f>D7*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2148,7 +2087,7 @@
         <f>E7+(D8*414)</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="18">
         <f>F7*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2156,19 +2095,19 @@
         <f>G7+(F8*414)</f>
         <v/>
       </c>
-      <c r="H8" s="33" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹949 Net)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Month 4</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="18">
         <f>B8*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2176,7 +2115,7 @@
         <f>C8+(B9*914)</f>
         <v/>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="18">
         <f>D8*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2184,7 +2123,7 @@
         <f>E8+(D9*914)</f>
         <v/>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="18">
         <f>F8*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2192,19 +2131,19 @@
         <f>G8+(F9*914)</f>
         <v/>
       </c>
-      <c r="H9" s="33" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Month 5</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="18">
         <f>B9*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2212,7 +2151,7 @@
         <f>C9+(B10*914)</f>
         <v/>
       </c>
-      <c r="D10" s="32">
+      <c r="D10" s="18">
         <f>D9*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2220,7 +2159,7 @@
         <f>E9+(D10*914)</f>
         <v/>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="18">
         <f>F9*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2228,19 +2167,19 @@
         <f>G9+(F10*914)</f>
         <v/>
       </c>
-      <c r="H10" s="33" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Month 6</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="18">
         <f>B10*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2248,7 +2187,7 @@
         <f>C10+(B11*914)</f>
         <v/>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="18">
         <f>D10*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2256,27 +2195,27 @@
         <f>E10+(D11*914)</f>
         <v/>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="18">
         <f>F10*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="22">
         <f>G10+(F11*914)</f>
         <v/>
       </c>
-      <c r="H11" s="33" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Month 7</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="18">
         <f>B11*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2284,15 +2223,15 @@
         <f>C11+(B12*914)</f>
         <v/>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="18">
         <f>D11*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="E12" s="34">
+      <c r="E12" s="22">
         <f>E11+(D12*914)</f>
         <v/>
       </c>
-      <c r="F12" s="32">
+      <c r="F12" s="18">
         <f>F11*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2300,27 +2239,27 @@
         <f>G11+(F12*914)</f>
         <v/>
       </c>
-      <c r="H12" s="33" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Month 8</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="18">
         <f>B12*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C13" s="34">
+      <c r="C13" s="22">
         <f>C12+(B13*914)</f>
         <v/>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="18">
         <f>D12*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2328,7 +2267,7 @@
         <f>E12+(D13*914)</f>
         <v/>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="18">
         <f>F12*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2336,19 +2275,19 @@
         <f>G12+(F13*914)</f>
         <v/>
       </c>
-      <c r="H13" s="33" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Month 9</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="18">
         <f>B13*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2356,7 +2295,7 @@
         <f>C13+(B14*914)</f>
         <v/>
       </c>
-      <c r="D14" s="32">
+      <c r="D14" s="18">
         <f>D13*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2364,7 +2303,7 @@
         <f>E13+(D14*914)</f>
         <v/>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="18">
         <f>F13*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2372,19 +2311,19 @@
         <f>G13+(F14*914)</f>
         <v/>
       </c>
-      <c r="H14" s="33" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Month 10</t>
         </is>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="18">
         <f>B14*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2392,7 +2331,7 @@
         <f>C14+(B15*914)</f>
         <v/>
       </c>
-      <c r="D15" s="32">
+      <c r="D15" s="18">
         <f>D14*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2400,7 +2339,7 @@
         <f>E14+(D15*914)</f>
         <v/>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="18">
         <f>F14*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2408,19 +2347,19 @@
         <f>G14+(F15*914)</f>
         <v/>
       </c>
-      <c r="H15" s="33" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Month 11</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="18">
         <f>B15*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2428,7 +2367,7 @@
         <f>C15+(B16*914)</f>
         <v/>
       </c>
-      <c r="D16" s="32">
+      <c r="D16" s="18">
         <f>D15*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2436,7 +2375,7 @@
         <f>E15+(D16*914)</f>
         <v/>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="18">
         <f>F15*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2444,19 +2383,19 @@
         <f>G15+(F16*914)</f>
         <v/>
       </c>
-      <c r="H16" s="33" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Month 12</t>
         </is>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="18">
         <f>B16*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2464,7 +2403,7 @@
         <f>C16+(B17*914)</f>
         <v/>
       </c>
-      <c r="D17" s="32">
+      <c r="D17" s="18">
         <f>D16*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2472,7 +2411,7 @@
         <f>E16+(D17*914)</f>
         <v/>
       </c>
-      <c r="F17" s="32">
+      <c r="F17" s="18">
         <f>F16*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2480,19 +2419,19 @@
         <f>G16+(F17*914)</f>
         <v/>
       </c>
-      <c r="H17" s="33" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Month 13</t>
         </is>
       </c>
-      <c r="B18" s="32">
+      <c r="B18" s="18">
         <f>B17*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2500,7 +2439,7 @@
         <f>C17+(B18*914)</f>
         <v/>
       </c>
-      <c r="D18" s="32">
+      <c r="D18" s="18">
         <f>D17*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2508,7 +2447,7 @@
         <f>E17+(D18*914)</f>
         <v/>
       </c>
-      <c r="F18" s="32">
+      <c r="F18" s="18">
         <f>F17*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2516,19 +2455,19 @@
         <f>G17+(F18*914)</f>
         <v/>
       </c>
-      <c r="H18" s="33" t="inlineStr">
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Month 14</t>
         </is>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="18">
         <f>B18*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2536,7 +2475,7 @@
         <f>C18+(B19*914)</f>
         <v/>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="18">
         <f>D18*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2544,7 +2483,7 @@
         <f>E18+(D19*914)</f>
         <v/>
       </c>
-      <c r="F19" s="32">
+      <c r="F19" s="18">
         <f>F18*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2552,19 +2491,19 @@
         <f>G18+(F19*914)</f>
         <v/>
       </c>
-      <c r="H19" s="33" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Month 15</t>
         </is>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="18">
         <f>B19*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2572,7 +2511,7 @@
         <f>C19+(B20*914)</f>
         <v/>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="18">
         <f>D19*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2580,7 +2519,7 @@
         <f>E19+(D20*914)</f>
         <v/>
       </c>
-      <c r="F20" s="32">
+      <c r="F20" s="18">
         <f>F19*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2588,19 +2527,19 @@
         <f>G19+(F20*914)</f>
         <v/>
       </c>
-      <c r="H20" s="33" t="inlineStr">
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Month 16</t>
         </is>
       </c>
-      <c r="B21" s="32">
+      <c r="B21" s="18">
         <f>B20*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2608,7 +2547,7 @@
         <f>C20+(B21*914)</f>
         <v/>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="18">
         <f>D20*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2616,7 +2555,7 @@
         <f>E20+(D21*914)</f>
         <v/>
       </c>
-      <c r="F21" s="32">
+      <c r="F21" s="18">
         <f>F20*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2624,19 +2563,19 @@
         <f>G20+(F21*914)</f>
         <v/>
       </c>
-      <c r="H21" s="33" t="inlineStr">
+      <c r="H21" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Month 17</t>
         </is>
       </c>
-      <c r="B22" s="32">
+      <c r="B22" s="18">
         <f>B21*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2644,7 +2583,7 @@
         <f>C21+(B22*914)</f>
         <v/>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="18">
         <f>D21*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2652,7 +2591,7 @@
         <f>E21+(D22*914)</f>
         <v/>
       </c>
-      <c r="F22" s="32">
+      <c r="F22" s="18">
         <f>F21*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2660,19 +2599,19 @@
         <f>G21+(F22*914)</f>
         <v/>
       </c>
-      <c r="H22" s="33" t="inlineStr">
+      <c r="H22" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Month 18</t>
         </is>
       </c>
-      <c r="B23" s="32">
+      <c r="B23" s="18">
         <f>B22*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2680,7 +2619,7 @@
         <f>C22+(B23*914)</f>
         <v/>
       </c>
-      <c r="D23" s="32">
+      <c r="D23" s="18">
         <f>D22*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2688,7 +2627,7 @@
         <f>E22+(D23*914)</f>
         <v/>
       </c>
-      <c r="F23" s="32">
+      <c r="F23" s="18">
         <f>F22*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2696,19 +2635,19 @@
         <f>G22+(F23*914)</f>
         <v/>
       </c>
-      <c r="H23" s="33" t="inlineStr">
+      <c r="H23" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Month 19</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="18">
         <f>B23*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2716,7 +2655,7 @@
         <f>C23+(B24*914)</f>
         <v/>
       </c>
-      <c r="D24" s="32">
+      <c r="D24" s="18">
         <f>D23*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2724,7 +2663,7 @@
         <f>E23+(D24*914)</f>
         <v/>
       </c>
-      <c r="F24" s="32">
+      <c r="F24" s="18">
         <f>F23*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2732,19 +2671,19 @@
         <f>G23+(F24*914)</f>
         <v/>
       </c>
-      <c r="H24" s="33" t="inlineStr">
+      <c r="H24" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Month 20</t>
         </is>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="18">
         <f>B24*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2752,7 +2691,7 @@
         <f>C24+(B25*914)</f>
         <v/>
       </c>
-      <c r="D25" s="32">
+      <c r="D25" s="18">
         <f>D24*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2760,7 +2699,7 @@
         <f>E24+(D25*914)</f>
         <v/>
       </c>
-      <c r="F25" s="32">
+      <c r="F25" s="18">
         <f>F24*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2768,19 +2707,19 @@
         <f>G24+(F25*914)</f>
         <v/>
       </c>
-      <c r="H25" s="33" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Month 21</t>
         </is>
       </c>
-      <c r="B26" s="32">
+      <c r="B26" s="18">
         <f>B25*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2788,7 +2727,7 @@
         <f>C25+(B26*914)</f>
         <v/>
       </c>
-      <c r="D26" s="32">
+      <c r="D26" s="18">
         <f>D25*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2796,7 +2735,7 @@
         <f>E25+(D26*914)</f>
         <v/>
       </c>
-      <c r="F26" s="32">
+      <c r="F26" s="18">
         <f>F25*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2804,19 +2743,19 @@
         <f>G25+(F26*914)</f>
         <v/>
       </c>
-      <c r="H26" s="33" t="inlineStr">
+      <c r="H26" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Month 22</t>
         </is>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="18">
         <f>B26*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2824,7 +2763,7 @@
         <f>C26+(B27*914)</f>
         <v/>
       </c>
-      <c r="D27" s="32">
+      <c r="D27" s="18">
         <f>D26*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2832,7 +2771,7 @@
         <f>E26+(D27*914)</f>
         <v/>
       </c>
-      <c r="F27" s="32">
+      <c r="F27" s="18">
         <f>F26*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2840,19 +2779,19 @@
         <f>G26+(F27*914)</f>
         <v/>
       </c>
-      <c r="H27" s="33" t="inlineStr">
+      <c r="H27" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Month 23</t>
         </is>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="18">
         <f>B27*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2860,7 +2799,7 @@
         <f>C27+(B28*914)</f>
         <v/>
       </c>
-      <c r="D28" s="32">
+      <c r="D28" s="18">
         <f>D27*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2868,7 +2807,7 @@
         <f>E27+(D28*914)</f>
         <v/>
       </c>
-      <c r="F28" s="32">
+      <c r="F28" s="18">
         <f>F27*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2876,19 +2815,19 @@
         <f>G27+(F28*914)</f>
         <v/>
       </c>
-      <c r="H28" s="33" t="inlineStr">
+      <c r="H28" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Month 24</t>
         </is>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="18">
         <f>B28*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2896,7 +2835,7 @@
         <f>C28+(B29*914)</f>
         <v/>
       </c>
-      <c r="D29" s="32">
+      <c r="D29" s="18">
         <f>D28*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2904,7 +2843,7 @@
         <f>E28+(D29*914)</f>
         <v/>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="18">
         <f>F28*(1-(0.05/12))</f>
         <v/>
       </c>
@@ -2912,7 +2851,7 @@
         <f>G28+(F29*914)</f>
         <v/>
       </c>
-      <c r="H29" s="33" t="inlineStr">
+      <c r="H29" s="21" t="inlineStr">
         <is>
           <t>Standard pricing (₹1,449 Net)</t>
         </is>
@@ -3003,874 +2942,874 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Month 0 (Acquisition)</t>
         </is>
       </c>
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="20" t="n">
         <v>1000</v>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Ecosystem Setup &amp; CAC Outflow</t>
         </is>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="29" t="n">
+      <c r="E5" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="19">
         <f>B5*('Illustrative Cost Breakdown'!D9+'Illustrative Cost Breakdown'!D19)</f>
         <v/>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="19">
         <f>-F5</f>
         <v/>
       </c>
-      <c r="H5" s="29">
+      <c r="H5" s="19">
         <f>G5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="18">
         <f>B5*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹999/mo)</t>
         </is>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="19">
         <f>B6*(999-50)</f>
         <v/>
       </c>
-      <c r="E6" s="35">
+      <c r="E6" s="19">
         <f>B6*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F6" s="35" t="n">
+      <c r="F6" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="35">
+      <c r="G6" s="19">
         <f>D6-E6</f>
         <v/>
       </c>
-      <c r="H6" s="9">
+      <c r="H6" s="5">
         <f>H5+G6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="B7" s="32">
+      <c r="B7" s="18">
         <f>B6*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹999/mo)</t>
         </is>
       </c>
-      <c r="D7" s="35">
+      <c r="D7" s="19">
         <f>B7*(999-50)</f>
         <v/>
       </c>
-      <c r="E7" s="35">
+      <c r="E7" s="19">
         <f>B7*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F7" s="35" t="n">
+      <c r="F7" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="35">
+      <c r="G7" s="19">
         <f>D7-E7</f>
         <v/>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="5">
         <f>H6+G7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="B8" s="32">
+      <c r="B8" s="18">
         <f>B7*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>Promo Pricing (₹999/mo)</t>
         </is>
       </c>
-      <c r="D8" s="35">
+      <c r="D8" s="19">
         <f>B8*(999-50)</f>
         <v/>
       </c>
-      <c r="E8" s="35">
+      <c r="E8" s="19">
         <f>B8*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F8" s="35" t="n">
+      <c r="F8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="35">
+      <c r="G8" s="19">
         <f>D8-E8</f>
         <v/>
       </c>
-      <c r="H8" s="9">
+      <c r="H8" s="5">
         <f>H7+G8</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Month 4</t>
         </is>
       </c>
-      <c r="B9" s="32">
+      <c r="B9" s="18">
         <f>B8*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="19">
         <f>B9*(1499-50)</f>
         <v/>
       </c>
-      <c r="E9" s="35">
+      <c r="E9" s="19">
         <f>B9*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F9" s="35" t="n">
+      <c r="F9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="35">
+      <c r="G9" s="19">
         <f>D9-E9</f>
         <v/>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="5">
         <f>H8+G9</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Month 5</t>
         </is>
       </c>
-      <c r="B10" s="32">
+      <c r="B10" s="18">
         <f>B9*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D10" s="35">
+      <c r="D10" s="19">
         <f>B10*(1499-50)</f>
         <v/>
       </c>
-      <c r="E10" s="35">
+      <c r="E10" s="19">
         <f>B10*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F10" s="35" t="n">
+      <c r="F10" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="35">
+      <c r="G10" s="19">
         <f>D10-E10</f>
         <v/>
       </c>
-      <c r="H10" s="9">
+      <c r="H10" s="5">
         <f>H9+G10</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Month 6</t>
         </is>
       </c>
-      <c r="B11" s="32">
+      <c r="B11" s="18">
         <f>B10*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C11" s="33" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D11" s="35">
+      <c r="D11" s="19">
         <f>B11*(1499-50)</f>
         <v/>
       </c>
-      <c r="E11" s="35">
+      <c r="E11" s="19">
         <f>B11*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F11" s="35" t="n">
+      <c r="F11" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="35">
+      <c r="G11" s="19">
         <f>D11-E11</f>
         <v/>
       </c>
-      <c r="H11" s="9">
+      <c r="H11" s="5">
         <f>H10+G11</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="31" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Month 7</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="18">
         <f>B11*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D12" s="35">
+      <c r="D12" s="19">
         <f>B12*(1499-50)</f>
         <v/>
       </c>
-      <c r="E12" s="35">
+      <c r="E12" s="19">
         <f>B12*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F12" s="35" t="n">
+      <c r="F12" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="35">
+      <c r="G12" s="19">
         <f>D12-E12</f>
         <v/>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="5">
         <f>H11+G12</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Month 8</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="18">
         <f>B12*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D13" s="35">
+      <c r="D13" s="19">
         <f>B13*(1499-50)</f>
         <v/>
       </c>
-      <c r="E13" s="35">
+      <c r="E13" s="19">
         <f>B13*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F13" s="35" t="n">
+      <c r="F13" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="35">
+      <c r="G13" s="19">
         <f>D13-E13</f>
         <v/>
       </c>
-      <c r="H13" s="9">
+      <c r="H13" s="5">
         <f>H12+G13</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Month 9 (PAYBACK BREAK-EVEN)</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="18">
         <f>B13*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D14" s="35">
+      <c r="D14" s="19">
         <f>B14*(1499-50)</f>
         <v/>
       </c>
-      <c r="E14" s="35">
+      <c r="E14" s="19">
         <f>B14*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F14" s="35" t="n">
+      <c r="F14" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="35">
+      <c r="G14" s="19">
         <f>D14-E14</f>
         <v/>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="22">
         <f>H13+G14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Month 10</t>
         </is>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="18">
         <f>B14*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="19">
         <f>B15*(1499-50)</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="19">
         <f>B15*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F15" s="35" t="n">
+      <c r="F15" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="35">
+      <c r="G15" s="19">
         <f>D15-E15</f>
         <v/>
       </c>
-      <c r="H15" s="9">
+      <c r="H15" s="5">
         <f>H14+G15</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Month 11</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="18">
         <f>B15*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="19">
         <f>B16*(1499-50)</f>
         <v/>
       </c>
-      <c r="E16" s="35">
+      <c r="E16" s="19">
         <f>B16*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F16" s="35" t="n">
+      <c r="F16" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16" s="19">
         <f>D16-E16</f>
         <v/>
       </c>
-      <c r="H16" s="9">
+      <c r="H16" s="5">
         <f>H15+G16</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Month 12</t>
         </is>
       </c>
-      <c r="B17" s="32">
+      <c r="B17" s="18">
         <f>B16*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C17" s="33" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D17" s="35">
+      <c r="D17" s="19">
         <f>B17*(1499-50)</f>
         <v/>
       </c>
-      <c r="E17" s="35">
+      <c r="E17" s="19">
         <f>B17*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F17" s="35" t="n">
+      <c r="F17" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="35">
+      <c r="G17" s="19">
         <f>D17-E17</f>
         <v/>
       </c>
-      <c r="H17" s="9">
+      <c r="H17" s="5">
         <f>H16+G17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="31" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Month 13</t>
         </is>
       </c>
-      <c r="B18" s="32">
+      <c r="B18" s="18">
         <f>B17*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="19">
         <f>B18*(1499-50)</f>
         <v/>
       </c>
-      <c r="E18" s="35">
+      <c r="E18" s="19">
         <f>B18*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F18" s="35" t="n">
+      <c r="F18" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="35">
+      <c r="G18" s="19">
         <f>D18-E18</f>
         <v/>
       </c>
-      <c r="H18" s="9">
+      <c r="H18" s="5">
         <f>H17+G18</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Month 14</t>
         </is>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="18">
         <f>B18*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D19" s="35">
+      <c r="D19" s="19">
         <f>B19*(1499-50)</f>
         <v/>
       </c>
-      <c r="E19" s="35">
+      <c r="E19" s="19">
         <f>B19*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F19" s="35" t="n">
+      <c r="F19" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="19">
         <f>D19-E19</f>
         <v/>
       </c>
-      <c r="H19" s="9">
+      <c r="H19" s="5">
         <f>H18+G19</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Month 15</t>
         </is>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="18">
         <f>B19*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="19">
         <f>B20*(1499-50)</f>
         <v/>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="19">
         <f>B20*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F20" s="35" t="n">
+      <c r="F20" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="35">
+      <c r="G20" s="19">
         <f>D20-E20</f>
         <v/>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="5">
         <f>H19+G20</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Month 16</t>
         </is>
       </c>
-      <c r="B21" s="32">
+      <c r="B21" s="18">
         <f>B20*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D21" s="35">
+      <c r="D21" s="19">
         <f>B21*(1499-50)</f>
         <v/>
       </c>
-      <c r="E21" s="35">
+      <c r="E21" s="19">
         <f>B21*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F21" s="35" t="n">
+      <c r="F21" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="35">
+      <c r="G21" s="19">
         <f>D21-E21</f>
         <v/>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="5">
         <f>H20+G21</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Month 17</t>
         </is>
       </c>
-      <c r="B22" s="32">
+      <c r="B22" s="18">
         <f>B21*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D22" s="35">
+      <c r="D22" s="19">
         <f>B22*(1499-50)</f>
         <v/>
       </c>
-      <c r="E22" s="35">
+      <c r="E22" s="19">
         <f>B22*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F22" s="35" t="n">
+      <c r="F22" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="35">
+      <c r="G22" s="19">
         <f>D22-E22</f>
         <v/>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="5">
         <f>H21+G22</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Month 18</t>
         </is>
       </c>
-      <c r="B23" s="32">
+      <c r="B23" s="18">
         <f>B22*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="C23" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D23" s="35">
+      <c r="D23" s="19">
         <f>B23*(1499-50)</f>
         <v/>
       </c>
-      <c r="E23" s="35">
+      <c r="E23" s="19">
         <f>B23*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F23" s="35" t="n">
+      <c r="F23" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="35">
+      <c r="G23" s="19">
         <f>D23-E23</f>
         <v/>
       </c>
-      <c r="H23" s="9">
+      <c r="H23" s="5">
         <f>H22+G23</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Month 19</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="18">
         <f>B23*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C24" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D24" s="35">
+      <c r="D24" s="19">
         <f>B24*(1499-50)</f>
         <v/>
       </c>
-      <c r="E24" s="35">
+      <c r="E24" s="19">
         <f>B24*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F24" s="35" t="n">
+      <c r="F24" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="35">
+      <c r="G24" s="19">
         <f>D24-E24</f>
         <v/>
       </c>
-      <c r="H24" s="9">
+      <c r="H24" s="5">
         <f>H23+G24</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="31" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Month 20</t>
         </is>
       </c>
-      <c r="B25" s="32">
+      <c r="B25" s="18">
         <f>B24*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D25" s="35">
+      <c r="D25" s="19">
         <f>B25*(1499-50)</f>
         <v/>
       </c>
-      <c r="E25" s="35">
+      <c r="E25" s="19">
         <f>B25*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F25" s="35" t="n">
+      <c r="F25" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="35">
+      <c r="G25" s="19">
         <f>D25-E25</f>
         <v/>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="5">
         <f>H24+G25</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="31" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Month 21</t>
         </is>
       </c>
-      <c r="B26" s="32">
+      <c r="B26" s="18">
         <f>B25*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D26" s="35">
+      <c r="D26" s="19">
         <f>B26*(1499-50)</f>
         <v/>
       </c>
-      <c r="E26" s="35">
+      <c r="E26" s="19">
         <f>B26*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F26" s="35" t="n">
+      <c r="F26" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="35">
+      <c r="G26" s="19">
         <f>D26-E26</f>
         <v/>
       </c>
-      <c r="H26" s="9">
+      <c r="H26" s="5">
         <f>H25+G26</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Month 22</t>
         </is>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="18">
         <f>B26*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D27" s="35">
+      <c r="D27" s="19">
         <f>B27*(1499-50)</f>
         <v/>
       </c>
-      <c r="E27" s="35">
+      <c r="E27" s="19">
         <f>B27*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F27" s="35" t="n">
+      <c r="F27" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="35">
+      <c r="G27" s="19">
         <f>D27-E27</f>
         <v/>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="5">
         <f>H26+G27</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Month 23</t>
         </is>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="18">
         <f>B27*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C28" s="33" t="inlineStr">
+      <c r="C28" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D28" s="35">
+      <c r="D28" s="19">
         <f>B28*(1499-50)</f>
         <v/>
       </c>
-      <c r="E28" s="35">
+      <c r="E28" s="19">
         <f>B28*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F28" s="35" t="n">
+      <c r="F28" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="35">
+      <c r="G28" s="19">
         <f>D28-E28</f>
         <v/>
       </c>
-      <c r="H28" s="9">
+      <c r="H28" s="5">
         <f>H27+G28</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Month 24</t>
         </is>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="18">
         <f>B28*(1-(0.05/12))</f>
         <v/>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>Standard Bundle (₹1,499/mo)</t>
         </is>
       </c>
-      <c r="D29" s="35">
+      <c r="D29" s="19">
         <f>B29*(1499-50)</f>
         <v/>
       </c>
-      <c r="E29" s="35">
+      <c r="E29" s="19">
         <f>B29*'Illustrative Cost Breakdown'!B30</f>
         <v/>
       </c>
-      <c r="F29" s="35" t="n">
+      <c r="F29" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="35">
+      <c r="G29" s="19">
         <f>D29-E29</f>
         <v/>
       </c>
-      <c r="H29" s="9">
+      <c r="H29" s="5">
         <f>H28+G29</f>
         <v/>
       </c>
@@ -3878,25 +3817,25 @@
     <row r="30"/>
     <row r="31"/>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Development Cost Amortization</t>
         </is>
       </c>
-      <c r="B32" s="24">
+      <c r="B32" s="16">
         <f>-'Illustrative Cost Breakdown'!D5</f>
         <v/>
       </c>
-      <c r="C32" s="37" t="n"/>
-      <c r="D32" s="37" t="n"/>
-      <c r="E32" s="37" t="n"/>
-      <c r="F32" s="37" t="n"/>
-      <c r="G32" s="23" t="inlineStr">
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="15" t="inlineStr">
         <is>
           <t>Total Cohort Net Profit</t>
         </is>
       </c>
-      <c r="H32" s="24">
+      <c r="H32" s="16">
         <f>H29+B32</f>
         <v/>
       </c>
@@ -3968,110 +3907,110 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Altura Starter</t>
         </is>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="25" t="n">
         <v>499</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="10" t="n">
         <v>0.82</v>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="25">
         <f>B5*C5</f>
         <v/>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>High acceptance for entry-level; limited monetization capability</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Altura Connect</t>
         </is>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="25" t="n">
         <v>999</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="10" t="n">
         <v>0.68</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="25">
         <f>B6*C6</f>
         <v/>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Steady standard tier; good for couples and smaller households</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Family Secure (Promo)</t>
         </is>
       </c>
-      <c r="B7" s="40" t="n">
+      <c r="B7" s="27" t="n">
         <v>999</v>
       </c>
-      <c r="C7" s="41" t="n">
+      <c r="C7" s="28" t="n">
         <v>0.89</v>
       </c>
-      <c r="D7" s="42">
+      <c r="D7" s="27">
         <f>B7*C7</f>
         <v/>
       </c>
-      <c r="E7" s="43" t="inlineStr">
+      <c r="E7" s="26" t="inlineStr">
         <is>
           <t>OPTIMAL SWEET SPOT: Lifts acceptance by 111% vs. standard price</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Family Secure (Standard)</t>
         </is>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="25" t="n">
         <v>1499</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="10" t="n">
         <v>0.42</v>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="25">
         <f>B8*C8</f>
         <v/>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>High long-term ARPU but requires promo introductory hook to convert</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Altura Infinite</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="25" t="n">
         <v>2999</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="10" t="n">
         <v>0.15</v>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="25">
         <f>B9*C9</f>
         <v/>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Niche high-value play; generates premium ARPU from 15% of market</t>
         </is>
@@ -4109,110 +4048,110 @@
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>Core Convergence Offer</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Broadband + TV + OTT bundles</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Partnership-only (No owned Fiber)</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>Broadband + TV + Mobile SIMs + Bank + Security</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Entry Price Point</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>₹399/mo (standalone fiber)</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>N/A (mobile only)</t>
         </is>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>₹499/mo (Starter Bundle)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Home Security integration</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>JioFiber smart camera (unintegrated app)</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>No home security products</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Altura Xsafe camera with cellular failover backup</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Loyalty Rewards</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>JioPrime coupon tie-ups</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Vi Rewards app checkouts</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Altura Thanks Coins (integrated bill cashbacks)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Financial Integration</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>UPI Payments wallet</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>Paytm/Third-party tie-ups</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>Altura Payments Bank (7% interest &amp; Safe Pay)</t>
         </is>

</xml_diff>